<commit_message>
Waarderingskamer: Fullrespec standaard op "yes" gezet.
Minor.
</commit_message>
<xml_diff>
--- a/src/main/resources/input/Waarderingskamer/props/Waarderingskamer.xlsx
+++ b/src/main/resources/input/Waarderingskamer/props/Waarderingskamer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\gitprojects\Imvertor-Maven\src\main\resources\input\Waarderingskamer\props\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153B419E-7061-479A-8F6C-D8326AEA4B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C87F52-CA46-427A-AAE0-CCD71B495727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="2280" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="20057" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Waarderingskamer" sheetId="3" r:id="rId1"/>
@@ -3312,7 +3312,7 @@
         <v>1</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G57" s="16"/>
       <c r="L57" s="16"/>

</xml_diff>